<commit_message>
Añadir resumen_factores_completo.xlsx formato correcto
</commit_message>
<xml_diff>
--- a/TFM_mao/resultados/biological_analisis/resumen_factores_completo.xlsx
+++ b/TFM_mao/resultados/biological_analisis/resumen_factores_completo.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>F_concentration</t>
+          <t>F_statconcentration</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>F_drug</t>
+          <t>F_statdrug</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>F_moa_fine</t>
+          <t>F_statmoa_fine</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -530,7 +530,7 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>F_plate</t>
+          <t>F_statplate</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>F_concentration</t>
+          <t>F_statconcentration</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -5004,7 +5004,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>F_drug</t>
+          <t>F_statdrug</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>F_moa_fine</t>
+          <t>F_statmoa_fine</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -5044,7 +5044,7 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>F_plate</t>
+          <t>F_statplate</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion de resultados; añadidos los resultados de los heatmaps de moa, de hallmarks y de progeny
</commit_message>
<xml_diff>
--- a/TFM_mao/resultados/biological_analisis/resumen_factores_completo.xlsx
+++ b/TFM_mao/resultados/biological_analisis/resumen_factores_completo.xlsx
@@ -567,17 +567,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Trail (9.91), EGFR (4.82), p53 (3.72), PI3K (3.31), Estrogen (1.58)</t>
+          <t>Trail (4.81), EGFR (2.12)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JAK-STAT (-6.59), Hypoxia (-5.49), VEGF (-3.12), Androgen (-2.82), TGFb (-2.10)</t>
+          <t>Hypoxia (-6.34), JAK-STAT (-6.19), MAPK (-2.42)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>HALLMARK_COAGULATION (4.04), HALLMARK_MYOGENESIS (3.20), HALLMARK_COMPLEMENT (2.86), HALLMARK_ALLOGRAFT_REJECTION (1.79), HALLMARK_SPERMATOGENESIS (1.12)</t>
+          <t>HALLMARK_COAGULATION (4.04), HALLMARK_MYOGENESIS (3.20), HALLMARK_COMPLEMENT (2.86), HALLMARK_ALLOGRAFT_REJECTION (1.79)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Hypoxia (18.62), JAK-STAT (12.23), Trail (3.12), WNT (1.21), TGFb (-0.56)</t>
+          <t>Hypoxia (13.79), JAK-STAT (11.85)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>NFkB (-10.36), TNFa (-9.04), PI3K (-8.77), MAPK (-6.61), EGFR (-5.13)</t>
+          <t>NFkB (-10.54), TNFa (-7.97), PI3K (-4.46), p53 (-2.57)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -753,12 +753,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EGFR (6.49), VEGF (4.72), MAPK (4.62), TGFb (1.46), p53 (1.04)</t>
+          <t>VEGF (4.14), EGFR (3.62)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>JAK-STAT (-5.27), WNT (-4.21), NFkB (-2.75), Trail (-2.61), TNFa (-2.48)</t>
+          <t>JAK-STAT (-4.61), NFkB (-2.52), WNT (-2.42), TNFa (-1.98)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -846,12 +846,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>JAK-STAT (5.34), p53 (4.01), Trail (2.53), TGFb (1.93), EGFR (0.13)</t>
+          <t>JAK-STAT (4.93), TGFb (2.75)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PI3K (-10.40), MAPK (-9.97), NFkB (-8.78), TNFa (-8.20), VEGF (-6.15)</t>
+          <t>NFkB (-7.64), TNFa (-6.29), MAPK (-5.84), PI3K (-4.86), Hypoxia (-3.88)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -937,19 +937,15 @@
           <t>PHLDA2 (-0.18), DUSP6 (-0.18), TMEM158 (-0.18), FOSL1 (-0.17), MT2A (-0.16), PPP1R14B (-0.16), S100A16 (-0.15), MIF (-0.15), IER3 (-0.15), G0S2 (-0.15)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>p53 (4.07), Trail (4.05), Androgen (-1.68), WNT (-1.71), JAK-STAT (-1.75)</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>MAPK (-23.60), EGFR (-21.96), TNFa (-13.13), NFkB (-12.15), Hypoxia (-9.87)</t>
+          <t>MAPK (-15.28), EGFR (-12.82), Hypoxia (-10.72), TNFa (-10.32), NFkB (-9.48)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>HALLMARK_BILE_ACID_METABOLISM (4.13), HALLMARK_ALLOGRAFT_REJECTION (3.02), HALLMARK_PI3K_AKT_MTOR_SIGNALING (2.69), HALLMARK_COMPLEMENT (1.69), HALLMARK_TGF_BETA_SIGNALING (1.25)</t>
+          <t>HALLMARK_BILE_ACID_METABOLISM (4.13), HALLMARK_ALLOGRAFT_REJECTION (3.02), HALLMARK_PI3K_AKT_MTOR_SIGNALING (2.69), HALLMARK_COMPLEMENT (1.69)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1032,17 +1028,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Hypoxia (1.96), Androgen (1.43), Estrogen (1.09), VEGF (0.59), Trail (-0.16)</t>
+          <t>Hypoxia (3.47), VEGF (2.60), Androgen (2.08)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>JAK-STAT (-14.91), NFkB (-13.51), TNFa (-12.69), PI3K (-4.70), EGFR (-4.55)</t>
+          <t>JAK-STAT (-14.70), NFkB (-8.03), TNFa (-8.01), PI3K (-3.31), MAPK (-2.65)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>HALLMARK_ADIPOGENESIS (5.53), HALLMARK_OXIDATIVE_PHOSPHORYLATION (5.08), HALLMARK_FATTY_ACID_METABOLISM (3.20), HALLMARK_ESTROGEN_RESPONSE_LATE (3.05), HALLMARK_SPERMATOGENESIS (2.56)</t>
+          <t>HALLMARK_ADIPOGENESIS (5.53), HALLMARK_OXIDATIVE_PHOSPHORYLATION (5.08), HALLMARK_FATTY_ACID_METABOLISM (3.20), HALLMARK_ESTROGEN_RESPONSE_LATE (3.05), HALLMARK_PEROXISOME (2.56)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1125,12 +1121,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>JAK-STAT (25.52), NFkB (13.01), TNFa (11.63), WNT (2.74), Trail (-0.09)</t>
+          <t>JAK-STAT (22.51), NFkB (9.41), TNFa (8.68), p53 (2.43)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MAPK (-10.15), Hypoxia (-8.81), EGFR (-7.16), PI3K (-5.57), Estrogen (-1.63)</t>
+          <t>MAPK (-5.84), Hypoxia (-4.60), PI3K (-2.46), EGFR (-2.45)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1218,12 +1214,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MAPK (32.59), EGFR (25.06), PI3K (9.29), Estrogen (7.30), VEGF (4.07)</t>
+          <t>MAPK (24.39), EGFR (15.54), PI3K (4.10), Estrogen (2.71)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Hypoxia (-12.60), JAK-STAT (-9.85), TNFa (-8.97), p53 (-8.70), NFkB (-8.18)</t>
+          <t>Hypoxia (-8.26), JAK-STAT (-7.77), NFkB (-5.98), TNFa (-5.96), p53 (-3.98)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1311,12 +1307,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hypoxia (16.10), Trail (3.63), Androgen (3.13), NFkB (0.50), p53 (0.14)</t>
+          <t>Hypoxia (9.36)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MAPK (-8.31), EGFR (-4.94), JAK-STAT (-3.27), PI3K (-3.12), WNT (-2.65)</t>
+          <t>JAK-STAT (-4.73), PI3K (-2.63), VEGF (-2.09)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1404,12 +1400,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NFkB (22.46), TNFa (21.12), EGFR (15.18), MAPK (14.42), Hypoxia (8.72)</t>
+          <t>NFkB (17.36), MAPK (15.69), TNFa (15.36), EGFR (13.24), TGFb (5.03)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PI3K (-9.74), WNT (-1.95), Estrogen (-1.92), Androgen (1.63), VEGF (2.18)</t>
+          <t>PI3K (-3.59)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1497,12 +1493,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NFkB (12.08), TNFa (10.93), TGFb (3.70), Hypoxia (3.00), PI3K (2.16)</t>
+          <t>NFkB (10.68), TNFa (9.48), TGFb (4.70), Androgen (3.15)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>p53 (-12.55), VEGF (-2.93), JAK-STAT (-1.85), WNT (-0.50), Estrogen (-0.47)</t>
+          <t>p53 (-7.09)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1590,12 +1586,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Hypoxia (10.31), NFkB (3.02), p53 (2.84), Trail (2.54), TNFa (2.32)</t>
+          <t>Hypoxia (3.74), NFkB (2.52), p53 (2.16)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>EGFR (-11.77), MAPK (-9.39), PI3K (-8.60), VEGF (-3.55), Estrogen (-3.03)</t>
+          <t>PI3K (-4.09), EGFR (-3.64), MAPK (-2.93)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1605,7 +1601,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>HALLMARK_OXIDATIVE_PHOSPHORYLATION (11.22), HALLMARK_MYC_TARGETS_V1 (9.85), HALLMARK_MYC_TARGETS_V2 (6.65), HALLMARK_UNFOLDED_PROTEIN_RESPONSE (4.45), HALLMARK_FATTY_ACID_METABOLISM (4.45)</t>
+          <t>HALLMARK_OXIDATIVE_PHOSPHORYLATION (11.22), HALLMARK_MYC_TARGETS_V1 (9.85), HALLMARK_MYC_TARGETS_V2 (6.65), HALLMARK_FATTY_ACID_METABOLISM (4.45), HALLMARK_UNFOLDED_PROTEIN_RESPONSE (4.45)</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -1683,12 +1679,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PI3K (6.30), p53 (3.54), WNT (2.46), VEGF (1.46), Estrogen (1.42)</t>
+          <t>PI3K (3.30)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>JAK-STAT (-5.21), Hypoxia (-4.30), NFkB (-1.75), MAPK (-1.72), TNFa (-1.38)</t>
+          <t>JAK-STAT (-4.48), MAPK (-2.89), Hypoxia (-2.75), TNFa (-2.23)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1776,12 +1772,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Androgen (9.10), MAPK (5.59), WNT (3.05), Estrogen (2.52), EGFR (-1.43)</t>
+          <t>Androgen (5.90), MAPK (4.86)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>JAK-STAT (-24.97), NFkB (-11.31), TNFa (-10.03), Hypoxia (-9.71), PI3K (-6.45)</t>
+          <t>JAK-STAT (-22.10), Hypoxia (-6.87), NFkB (-5.79), TNFa (-4.17), PI3K (-3.41)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1869,12 +1865,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>JAK-STAT (8.89), Trail (2.15), VEGF (0.87), TGFb (0.71), Androgen (-0.21)</t>
+          <t>JAK-STAT (7.72)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MAPK (-8.38), PI3K (-4.35), EGFR (-4.15), Estrogen (-2.70), p53 (-1.52)</t>
+          <t>MAPK (-5.04), EGFR (-4.73), NFkB (-3.17), p53 (-3.13), PI3K (-2.34)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1962,12 +1958,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>JAK-STAT (18.08), Hypoxia (8.48), p53 (2.29), VEGF (1.42), PI3K (1.03)</t>
+          <t>JAK-STAT (16.66), Hypoxia (8.12), p53 (3.48)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>EGFR (-7.34), MAPK (-6.21), TGFb (-4.70), Estrogen (-1.58), TNFa (-1.42)</t>
+          <t>MAPK (-5.62), EGFR (-4.55), TGFb (-2.46)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2055,12 +2051,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TNFa (2.54), NFkB (2.06), p53 (-0.05), VEGF (-0.92), TGFb (-1.07)</t>
+          <t>NFkB (2.48), TNFa (2.17)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>JAK-STAT (-11.28), PI3K (-3.97), MAPK (-3.56), EGFR (-3.35), Hypoxia (-2.33)</t>
+          <t>JAK-STAT (-11.66), Hypoxia (-3.78), EGFR (-3.56), PI3K (-3.27), MAPK (-2.93)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2148,12 +2144,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PI3K (8.87), EGFR (3.97), TGFb (3.96), Trail (2.14), Hypoxia (1.70)</t>
+          <t>PI3K (3.27), TGFb (3.02)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>JAK-STAT (-6.98), NFkB (-6.80), TNFa (-6.70), VEGF (-3.13), p53 (-2.67)</t>
+          <t>JAK-STAT (-6.92), MAPK (-6.59), NFkB (-6.39), p53 (-6.25), TNFa (-6.09)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2241,12 +2237,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>p53 (9.55), TNFa (3.72), NFkB (2.74), Trail (2.52), TGFb (0.90)</t>
+          <t>MAPK (5.84), NFkB (3.94), TNFa (3.52), p53 (3.01), TGFb (2.30)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>JAK-STAT (-17.79), PI3K (-15.62), Hypoxia (-6.87), Estrogen (-4.63), EGFR (-3.76)</t>
+          <t>JAK-STAT (-17.07), PI3K (-8.92), Hypoxia (-7.02), Estrogen (-2.17)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2334,14 +2330,10 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Hypoxia (28.64), JAK-STAT (28.06), NFkB (19.86), TNFa (18.03), PI3K (9.28)</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>VEGF (-1.23), WNT (-1.09), MAPK (-0.53), Trail (0.22), Estrogen (1.33)</t>
-        </is>
-      </c>
+          <t>JAK-STAT (25.51), Hypoxia (22.71), NFkB (13.31), TNFa (13.15), PI3K (4.86)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>HALLMARK_HYPOXIA (37.71), HALLMARK_TNFA_SIGNALING_VIA_NFKB (25.57), HALLMARK_INTERFERON_GAMMA_RESPONSE (15.60), HALLMARK_EPITHELIAL_MESENCHYMAL_TRANSITION (13.77), HALLMARK_P53_PATHWAY (13.70)</t>
@@ -2427,17 +2419,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>NFkB (12.26), TNFa (11.66), p53 (8.40), JAK-STAT (7.36), VEGF (3.58)</t>
+          <t>NFkB (8.29), TNFa (8.21), JAK-STAT (6.75), p53 (4.53), PI3K (3.00)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MAPK (-2.29), Estrogen (-1.19), Androgen (-0.82), TGFb (1.96), Hypoxia (2.04)</t>
+          <t>MAPK (-3.62)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>HALLMARK_TNFA_SIGNALING_VIA_NFKB (7.16), HALLMARK_INFLAMMATORY_RESPONSE (7.03), HALLMARK_KRAS_SIGNALING_UP (7.03), HALLMARK_HYPOXIA (6.64), HALLMARK_APOPTOSIS (5.29)</t>
+          <t>HALLMARK_TNFA_SIGNALING_VIA_NFKB (7.16), HALLMARK_KRAS_SIGNALING_UP (7.03), HALLMARK_INFLAMMATORY_RESPONSE (7.03), HALLMARK_HYPOXIA (6.64), HALLMARK_APOPTOSIS (5.29)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2518,14 +2510,10 @@
           <t>CFAP210 (-0.32), FOSB (-0.30), IQCN (-0.25), FGF18 (-0.25), FRMD5 (-0.23), RPS7 (-0.23), MLF1 (-0.21), CMSS1 (-0.21), TNFAIP3 (-0.21), TFRC (-0.21)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>TGFb (1.87), Androgen (-0.47), Trail (-0.51), VEGF (-1.08), Hypoxia (-1.39)</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MAPK (-13.22), EGFR (-10.92), NFkB (-9.66), TNFa (-9.33), PI3K (-8.31)</t>
+          <t>NFkB (-10.03), TNFa (-9.04), EGFR (-6.95), PI3K (-6.79), MAPK (-5.36)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2613,12 +2601,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Hypoxia (8.04), p53 (3.95), Androgen (3.82), Trail (3.67), TGFb (-1.10)</t>
+          <t>Hypoxia (4.96), Androgen (2.31)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>JAK-STAT (-14.20), PI3K (-8.88), NFkB (-8.77), TNFa (-7.45), MAPK (-6.29)</t>
+          <t>JAK-STAT (-14.32), NFkB (-6.82), TNFa (-6.49), PI3K (-5.57), WNT (-2.50)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2706,12 +2694,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>p53 (11.08), Hypoxia (6.57), Trail (4.38), EGFR (4.24), MAPK (3.06)</t>
+          <t>MAPK (7.94), p53 (4.49), Hypoxia (4.24), EGFR (3.76), TGFb (3.15)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>JAK-STAT (-13.54), Estrogen (-3.22), VEGF (-1.67), PI3K (-0.99), Androgen (0.44)</t>
+          <t>JAK-STAT (-14.45), VEGF (-2.89)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2799,12 +2787,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>JAK-STAT (36.75), p53 (16.41), NFkB (11.68), TNFa (8.54), EGFR (3.22)</t>
+          <t>JAK-STAT (33.96), p53 (8.09), NFkB (7.63), TNFa (5.45), VEGF (3.18)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Hypoxia (-9.92), TGFb (-4.49), WNT (-1.95), Androgen (-1.24), Trail (-1.19)</t>
+          <t>Hypoxia (-6.68), TGFb (-3.38)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2892,12 +2880,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>JAK-STAT (22.03), NFkB (21.34), TNFa (20.40), Androgen (3.55), TGFb (3.00)</t>
+          <t>JAK-STAT (20.14), NFkB (17.30), TNFa (16.61), Androgen (3.56), MAPK (2.95)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Hypoxia (-14.60), p53 (-3.89), VEGF (-1.88), Estrogen (0.29), WNT (0.38)</t>
+          <t>Hypoxia (-14.06), VEGF (-2.31), p53 (-2.30)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2985,12 +2973,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>EGFR (4.32), PI3K (3.92), Estrogen (0.98), MAPK (0.75), WNT (0.34)</t>
+          <t>EGFR (3.74), PI3K (2.54)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>JAK-STAT (-13.24), p53 (-3.25), TNFa (-2.73), NFkB (-2.10), VEGF (-0.72)</t>
+          <t>JAK-STAT (-12.29), p53 (-2.64)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3078,12 +3066,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>JAK-STAT (41.63), NFkB (11.63), TNFa (9.98), MAPK (4.90), Androgen (3.26)</t>
+          <t>JAK-STAT (39.72), NFkB (7.25), TNFa (6.55), Androgen (2.54)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>p53 (-7.03), Hypoxia (-2.57), Trail (-1.57), PI3K (-1.27), WNT (-0.16)</t>
+          <t>p53 (-2.54)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3171,14 +3159,10 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Hypoxia (9.33), JAK-STAT (6.76), NFkB (6.63), TNFa (6.43), EGFR (3.70)</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>PI3K (-1.37), Trail (-1.05), MAPK (-0.24), WNT (0.00), VEGF (0.86)</t>
-        </is>
-      </c>
+          <t>JAK-STAT (7.67), Hypoxia (7.62), NFkB (5.02), TNFa (4.76), EGFR (3.49)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>HALLMARK_HYPOXIA (12.36), HALLMARK_MTORC1_SIGNALING (9.63), HALLMARK_UNFOLDED_PROTEIN_RESPONSE (9.09), HALLMARK_GLYCOLYSIS (8.00), HALLMARK_P53_PATHWAY (7.46)</t>
@@ -3264,12 +3248,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Hypoxia (12.03), JAK-STAT (9.10), p53 (7.74), NFkB (2.84), TNFa (2.24)</t>
+          <t>Hypoxia (12.28), JAK-STAT (8.94), p53 (6.28), NFkB (2.08), PI3K (1.99)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>MAPK (-4.38), TGFb (-4.24), EGFR (-2.47), VEGF (-1.29), Estrogen (-0.03)</t>
+          <t>TGFb (-4.52), MAPK (-2.71)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3919,12 +3903,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Trail (9.91), EGFR (4.82), p53 (3.72), PI3K (3.31), Estrogen (1.58)</t>
+          <t>Trail (4.81), EGFR (2.12)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>JAK-STAT (-6.59), Hypoxia (-5.49), VEGF (-3.12), Androgen (-2.82), TGFb (-2.10)</t>
+          <t>Hypoxia (-6.34), JAK-STAT (-6.19), MAPK (-2.42)</t>
         </is>
       </c>
     </row>
@@ -3936,12 +3920,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hypoxia (18.62), JAK-STAT (12.23), Trail (3.12), WNT (1.21), TGFb (-0.56)</t>
+          <t>Hypoxia (13.79), JAK-STAT (11.85)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NFkB (-10.36), TNFa (-9.04), PI3K (-8.77), MAPK (-6.61), EGFR (-5.13)</t>
+          <t>NFkB (-10.54), TNFa (-7.97), PI3K (-4.46), p53 (-2.57)</t>
         </is>
       </c>
     </row>
@@ -3953,12 +3937,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EGFR (6.49), VEGF (4.72), MAPK (4.62), TGFb (1.46), p53 (1.04)</t>
+          <t>VEGF (4.14), EGFR (3.62)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>JAK-STAT (-5.27), WNT (-4.21), NFkB (-2.75), Trail (-2.61), TNFa (-2.48)</t>
+          <t>JAK-STAT (-4.61), NFkB (-2.52), WNT (-2.42), TNFa (-1.98)</t>
         </is>
       </c>
     </row>
@@ -3970,12 +3954,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JAK-STAT (5.34), p53 (4.01), Trail (2.53), TGFb (1.93), EGFR (0.13)</t>
+          <t>JAK-STAT (4.93), TGFb (2.75)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PI3K (-10.40), MAPK (-9.97), NFkB (-8.78), TNFa (-8.20), VEGF (-6.15)</t>
+          <t>NFkB (-7.64), TNFa (-6.29), MAPK (-5.84), PI3K (-4.86), Hypoxia (-3.88)</t>
         </is>
       </c>
     </row>
@@ -3985,14 +3969,10 @@
           <t>Factor5</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>p53 (4.07), Trail (4.05), Androgen (-1.68), WNT (-1.71), JAK-STAT (-1.75)</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MAPK (-23.60), EGFR (-21.96), TNFa (-13.13), NFkB (-12.15), Hypoxia (-9.87)</t>
+          <t>MAPK (-15.28), EGFR (-12.82), Hypoxia (-10.72), TNFa (-10.32), NFkB (-9.48)</t>
         </is>
       </c>
     </row>
@@ -4004,12 +3984,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hypoxia (1.96), Androgen (1.43), Estrogen (1.09), VEGF (0.59), Trail (-0.16)</t>
+          <t>Hypoxia (3.47), VEGF (2.60), Androgen (2.08)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>JAK-STAT (-14.91), NFkB (-13.51), TNFa (-12.69), PI3K (-4.70), EGFR (-4.55)</t>
+          <t>JAK-STAT (-14.70), NFkB (-8.03), TNFa (-8.01), PI3K (-3.31), MAPK (-2.65)</t>
         </is>
       </c>
     </row>
@@ -4021,12 +4001,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>JAK-STAT (25.52), NFkB (13.01), TNFa (11.63), WNT (2.74), Trail (-0.09)</t>
+          <t>JAK-STAT (22.51), NFkB (9.41), TNFa (8.68), p53 (2.43)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MAPK (-10.15), Hypoxia (-8.81), EGFR (-7.16), PI3K (-5.57), Estrogen (-1.63)</t>
+          <t>MAPK (-5.84), Hypoxia (-4.60), PI3K (-2.46), EGFR (-2.45)</t>
         </is>
       </c>
     </row>
@@ -4038,12 +4018,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MAPK (32.59), EGFR (25.06), PI3K (9.29), Estrogen (7.30), VEGF (4.07)</t>
+          <t>MAPK (24.39), EGFR (15.54), PI3K (4.10), Estrogen (2.71)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hypoxia (-12.60), JAK-STAT (-9.85), TNFa (-8.97), p53 (-8.70), NFkB (-8.18)</t>
+          <t>Hypoxia (-8.26), JAK-STAT (-7.77), NFkB (-5.98), TNFa (-5.96), p53 (-3.98)</t>
         </is>
       </c>
     </row>
@@ -4055,12 +4035,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hypoxia (16.10), Trail (3.63), Androgen (3.13), NFkB (0.50), p53 (0.14)</t>
+          <t>Hypoxia (9.36)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MAPK (-8.31), EGFR (-4.94), JAK-STAT (-3.27), PI3K (-3.12), WNT (-2.65)</t>
+          <t>JAK-STAT (-4.73), PI3K (-2.63), VEGF (-2.09)</t>
         </is>
       </c>
     </row>
@@ -4072,12 +4052,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NFkB (22.46), TNFa (21.12), EGFR (15.18), MAPK (14.42), Hypoxia (8.72)</t>
+          <t>NFkB (17.36), MAPK (15.69), TNFa (15.36), EGFR (13.24), TGFb (5.03)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PI3K (-9.74), WNT (-1.95), Estrogen (-1.92), Androgen (1.63), VEGF (2.18)</t>
+          <t>PI3K (-3.59)</t>
         </is>
       </c>
     </row>
@@ -4089,12 +4069,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NFkB (12.08), TNFa (10.93), TGFb (3.70), Hypoxia (3.00), PI3K (2.16)</t>
+          <t>NFkB (10.68), TNFa (9.48), TGFb (4.70), Androgen (3.15)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>p53 (-12.55), VEGF (-2.93), JAK-STAT (-1.85), WNT (-0.50), Estrogen (-0.47)</t>
+          <t>p53 (-7.09)</t>
         </is>
       </c>
     </row>
@@ -4106,12 +4086,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hypoxia (10.31), NFkB (3.02), p53 (2.84), Trail (2.54), TNFa (2.32)</t>
+          <t>Hypoxia (3.74), NFkB (2.52), p53 (2.16)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>EGFR (-11.77), MAPK (-9.39), PI3K (-8.60), VEGF (-3.55), Estrogen (-3.03)</t>
+          <t>PI3K (-4.09), EGFR (-3.64), MAPK (-2.93)</t>
         </is>
       </c>
     </row>
@@ -4123,12 +4103,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PI3K (6.30), p53 (3.54), WNT (2.46), VEGF (1.46), Estrogen (1.42)</t>
+          <t>PI3K (3.30)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>JAK-STAT (-5.21), Hypoxia (-4.30), NFkB (-1.75), MAPK (-1.72), TNFa (-1.38)</t>
+          <t>JAK-STAT (-4.48), MAPK (-2.89), Hypoxia (-2.75), TNFa (-2.23)</t>
         </is>
       </c>
     </row>
@@ -4140,12 +4120,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Androgen (9.10), MAPK (5.59), WNT (3.05), Estrogen (2.52), EGFR (-1.43)</t>
+          <t>Androgen (5.90), MAPK (4.86)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>JAK-STAT (-24.97), NFkB (-11.31), TNFa (-10.03), Hypoxia (-9.71), PI3K (-6.45)</t>
+          <t>JAK-STAT (-22.10), Hypoxia (-6.87), NFkB (-5.79), TNFa (-4.17), PI3K (-3.41)</t>
         </is>
       </c>
     </row>
@@ -4157,12 +4137,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>JAK-STAT (8.89), Trail (2.15), VEGF (0.87), TGFb (0.71), Androgen (-0.21)</t>
+          <t>JAK-STAT (7.72)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MAPK (-8.38), PI3K (-4.35), EGFR (-4.15), Estrogen (-2.70), p53 (-1.52)</t>
+          <t>MAPK (-5.04), EGFR (-4.73), NFkB (-3.17), p53 (-3.13), PI3K (-2.34)</t>
         </is>
       </c>
     </row>
@@ -4174,12 +4154,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>JAK-STAT (18.08), Hypoxia (8.48), p53 (2.29), VEGF (1.42), PI3K (1.03)</t>
+          <t>JAK-STAT (16.66), Hypoxia (8.12), p53 (3.48)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EGFR (-7.34), MAPK (-6.21), TGFb (-4.70), Estrogen (-1.58), TNFa (-1.42)</t>
+          <t>MAPK (-5.62), EGFR (-4.55), TGFb (-2.46)</t>
         </is>
       </c>
     </row>
@@ -4191,12 +4171,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TNFa (2.54), NFkB (2.06), p53 (-0.05), VEGF (-0.92), TGFb (-1.07)</t>
+          <t>NFkB (2.48), TNFa (2.17)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>JAK-STAT (-11.28), PI3K (-3.97), MAPK (-3.56), EGFR (-3.35), Hypoxia (-2.33)</t>
+          <t>JAK-STAT (-11.66), Hypoxia (-3.78), EGFR (-3.56), PI3K (-3.27), MAPK (-2.93)</t>
         </is>
       </c>
     </row>
@@ -4208,12 +4188,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PI3K (8.87), EGFR (3.97), TGFb (3.96), Trail (2.14), Hypoxia (1.70)</t>
+          <t>PI3K (3.27), TGFb (3.02)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>JAK-STAT (-6.98), NFkB (-6.80), TNFa (-6.70), VEGF (-3.13), p53 (-2.67)</t>
+          <t>JAK-STAT (-6.92), MAPK (-6.59), NFkB (-6.39), p53 (-6.25), TNFa (-6.09)</t>
         </is>
       </c>
     </row>
@@ -4225,12 +4205,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>p53 (9.55), TNFa (3.72), NFkB (2.74), Trail (2.52), TGFb (0.90)</t>
+          <t>MAPK (5.84), NFkB (3.94), TNFa (3.52), p53 (3.01), TGFb (2.30)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JAK-STAT (-17.79), PI3K (-15.62), Hypoxia (-6.87), Estrogen (-4.63), EGFR (-3.76)</t>
+          <t>JAK-STAT (-17.07), PI3K (-8.92), Hypoxia (-7.02), Estrogen (-2.17)</t>
         </is>
       </c>
     </row>
@@ -4242,14 +4222,10 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Hypoxia (28.64), JAK-STAT (28.06), NFkB (19.86), TNFa (18.03), PI3K (9.28)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>VEGF (-1.23), WNT (-1.09), MAPK (-0.53), Trail (0.22), Estrogen (1.33)</t>
-        </is>
-      </c>
+          <t>JAK-STAT (25.51), Hypoxia (22.71), NFkB (13.31), TNFa (13.15), PI3K (4.86)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4259,12 +4235,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NFkB (12.26), TNFa (11.66), p53 (8.40), JAK-STAT (7.36), VEGF (3.58)</t>
+          <t>NFkB (8.29), TNFa (8.21), JAK-STAT (6.75), p53 (4.53), PI3K (3.00)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MAPK (-2.29), Estrogen (-1.19), Androgen (-0.82), TGFb (1.96), Hypoxia (2.04)</t>
+          <t>MAPK (-3.62)</t>
         </is>
       </c>
     </row>
@@ -4274,14 +4250,10 @@
           <t>Factor22</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>TGFb (1.87), Androgen (-0.47), Trail (-0.51), VEGF (-1.08), Hypoxia (-1.39)</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MAPK (-13.22), EGFR (-10.92), NFkB (-9.66), TNFa (-9.33), PI3K (-8.31)</t>
+          <t>NFkB (-10.03), TNFa (-9.04), EGFR (-6.95), PI3K (-6.79), MAPK (-5.36)</t>
         </is>
       </c>
     </row>
@@ -4293,12 +4265,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Hypoxia (8.04), p53 (3.95), Androgen (3.82), Trail (3.67), TGFb (-1.10)</t>
+          <t>Hypoxia (4.96), Androgen (2.31)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>JAK-STAT (-14.20), PI3K (-8.88), NFkB (-8.77), TNFa (-7.45), MAPK (-6.29)</t>
+          <t>JAK-STAT (-14.32), NFkB (-6.82), TNFa (-6.49), PI3K (-5.57), WNT (-2.50)</t>
         </is>
       </c>
     </row>
@@ -4310,12 +4282,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>p53 (11.08), Hypoxia (6.57), Trail (4.38), EGFR (4.24), MAPK (3.06)</t>
+          <t>MAPK (7.94), p53 (4.49), Hypoxia (4.24), EGFR (3.76), TGFb (3.15)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>JAK-STAT (-13.54), Estrogen (-3.22), VEGF (-1.67), PI3K (-0.99), Androgen (0.44)</t>
+          <t>JAK-STAT (-14.45), VEGF (-2.89)</t>
         </is>
       </c>
     </row>
@@ -4327,12 +4299,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JAK-STAT (36.75), p53 (16.41), NFkB (11.68), TNFa (8.54), EGFR (3.22)</t>
+          <t>JAK-STAT (33.96), p53 (8.09), NFkB (7.63), TNFa (5.45), VEGF (3.18)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hypoxia (-9.92), TGFb (-4.49), WNT (-1.95), Androgen (-1.24), Trail (-1.19)</t>
+          <t>Hypoxia (-6.68), TGFb (-3.38)</t>
         </is>
       </c>
     </row>
@@ -4344,12 +4316,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JAK-STAT (22.03), NFkB (21.34), TNFa (20.40), Androgen (3.55), TGFb (3.00)</t>
+          <t>JAK-STAT (20.14), NFkB (17.30), TNFa (16.61), Androgen (3.56), MAPK (2.95)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hypoxia (-14.60), p53 (-3.89), VEGF (-1.88), Estrogen (0.29), WNT (0.38)</t>
+          <t>Hypoxia (-14.06), VEGF (-2.31), p53 (-2.30)</t>
         </is>
       </c>
     </row>
@@ -4361,12 +4333,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EGFR (4.32), PI3K (3.92), Estrogen (0.98), MAPK (0.75), WNT (0.34)</t>
+          <t>EGFR (3.74), PI3K (2.54)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>JAK-STAT (-13.24), p53 (-3.25), TNFa (-2.73), NFkB (-2.10), VEGF (-0.72)</t>
+          <t>JAK-STAT (-12.29), p53 (-2.64)</t>
         </is>
       </c>
     </row>
@@ -4378,12 +4350,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JAK-STAT (41.63), NFkB (11.63), TNFa (9.98), MAPK (4.90), Androgen (3.26)</t>
+          <t>JAK-STAT (39.72), NFkB (7.25), TNFa (6.55), Androgen (2.54)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>p53 (-7.03), Hypoxia (-2.57), Trail (-1.57), PI3K (-1.27), WNT (-0.16)</t>
+          <t>p53 (-2.54)</t>
         </is>
       </c>
     </row>
@@ -4395,14 +4367,10 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hypoxia (9.33), JAK-STAT (6.76), NFkB (6.63), TNFa (6.43), EGFR (3.70)</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>PI3K (-1.37), Trail (-1.05), MAPK (-0.24), WNT (0.00), VEGF (0.86)</t>
-        </is>
-      </c>
+          <t>JAK-STAT (7.67), Hypoxia (7.62), NFkB (5.02), TNFa (4.76), EGFR (3.49)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4412,12 +4380,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Hypoxia (12.03), JAK-STAT (9.10), p53 (7.74), NFkB (2.84), TNFa (2.24)</t>
+          <t>Hypoxia (12.28), JAK-STAT (8.94), p53 (6.28), NFkB (2.08), PI3K (1.99)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MAPK (-4.38), TGFb (-4.24), EGFR (-2.47), VEGF (-1.29), Estrogen (-0.03)</t>
+          <t>TGFb (-4.52), MAPK (-2.71)</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4428,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HALLMARK_COAGULATION (4.04), HALLMARK_MYOGENESIS (3.20), HALLMARK_COMPLEMENT (2.86), HALLMARK_ALLOGRAFT_REJECTION (1.79), HALLMARK_SPERMATOGENESIS (1.12)</t>
+          <t>HALLMARK_COAGULATION (4.04), HALLMARK_MYOGENESIS (3.20), HALLMARK_COMPLEMENT (2.86), HALLMARK_ALLOGRAFT_REJECTION (1.79)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4528,7 +4496,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HALLMARK_BILE_ACID_METABOLISM (4.13), HALLMARK_ALLOGRAFT_REJECTION (3.02), HALLMARK_PI3K_AKT_MTOR_SIGNALING (2.69), HALLMARK_COMPLEMENT (1.69), HALLMARK_TGF_BETA_SIGNALING (1.25)</t>
+          <t>HALLMARK_BILE_ACID_METABOLISM (4.13), HALLMARK_ALLOGRAFT_REJECTION (3.02), HALLMARK_PI3K_AKT_MTOR_SIGNALING (2.69), HALLMARK_COMPLEMENT (1.69)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4545,7 +4513,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HALLMARK_ADIPOGENESIS (5.53), HALLMARK_OXIDATIVE_PHOSPHORYLATION (5.08), HALLMARK_FATTY_ACID_METABOLISM (3.20), HALLMARK_ESTROGEN_RESPONSE_LATE (3.05), HALLMARK_SPERMATOGENESIS (2.56)</t>
+          <t>HALLMARK_ADIPOGENESIS (5.53), HALLMARK_OXIDATIVE_PHOSPHORYLATION (5.08), HALLMARK_FATTY_ACID_METABOLISM (3.20), HALLMARK_ESTROGEN_RESPONSE_LATE (3.05), HALLMARK_PEROXISOME (2.56)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4652,7 +4620,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HALLMARK_OXIDATIVE_PHOSPHORYLATION (11.22), HALLMARK_MYC_TARGETS_V1 (9.85), HALLMARK_MYC_TARGETS_V2 (6.65), HALLMARK_UNFOLDED_PROTEIN_RESPONSE (4.45), HALLMARK_FATTY_ACID_METABOLISM (4.45)</t>
+          <t>HALLMARK_OXIDATIVE_PHOSPHORYLATION (11.22), HALLMARK_MYC_TARGETS_V1 (9.85), HALLMARK_MYC_TARGETS_V2 (6.65), HALLMARK_FATTY_ACID_METABOLISM (4.45), HALLMARK_UNFOLDED_PROTEIN_RESPONSE (4.45)</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4768,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HALLMARK_TNFA_SIGNALING_VIA_NFKB (7.16), HALLMARK_INFLAMMATORY_RESPONSE (7.03), HALLMARK_KRAS_SIGNALING_UP (7.03), HALLMARK_HYPOXIA (6.64), HALLMARK_APOPTOSIS (5.29)</t>
+          <t>HALLMARK_TNFA_SIGNALING_VIA_NFKB (7.16), HALLMARK_KRAS_SIGNALING_UP (7.03), HALLMARK_INFLAMMATORY_RESPONSE (7.03), HALLMARK_HYPOXIA (6.64), HALLMARK_APOPTOSIS (5.29)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">

</xml_diff>